<commit_message>
modified data in excel
</commit_message>
<xml_diff>
--- a/guru99_automation/src/test/resources/testdata/CustomerId.xlsx
+++ b/guru99_automation/src/test/resources/testdata/CustomerId.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\wipro_capstone\guru99_capstone\guru99_automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E7B686-FC01-4E69-A2A4-27B319E96552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DCD218-30FF-4C8F-A1D2-3AEF96643170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4545" yWindow="1935" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4890" yWindow="2280" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CustomerID" sheetId="1" r:id="rId1"/>

</xml_diff>